<commit_message>
Update billing app features and templates for redeploy
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,10 +451,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Total (ex GST)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Payment Mode</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>User</t>
         </is>
@@ -482,9 +487,14 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>141.56</v>
+        <v>133.812</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -498,7 +508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KHUSHANSH</t>
+          <t>KUSHANSH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -512,11 +522,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>566.2</v>
+        <v>535.248</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
@@ -542,11 +557,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>125.4</v>
+        <v>118.818</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
@@ -572,11 +592,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>393.3</v>
+        <v>318.0375</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
@@ -602,9 +627,14 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>495</v>
+        <v>484.974</v>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -632,11 +662,16 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>365.4</v>
+        <v>343.35</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
@@ -662,18 +697,23 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>428.4</v>
+        <v>430.029</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INV-2026-1009</t>
+          <t>INV-2026-1008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -692,18 +732,23 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1448</v>
+        <v>1285.641</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>INV-2026-1010</t>
+          <t>INV-2026-1009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -722,23 +767,28 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1066.4</v>
+        <v>1045.791</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INV-2026-1011</t>
+          <t>INV-2026-1010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RAVINDER PAL SINGH</t>
+          <t>RAVINDRA PAL SINGH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -752,18 +802,23 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>411</v>
+        <v>369.4725</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INV-2026-1012</t>
+          <t>INV-2026-1011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -782,9 +837,14 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1472.4</v>
+        <v>1367.0028</v>
       </c>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -793,12 +853,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INV-2026-1014</t>
+          <t>INV-2026-1012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MANJU CHAUHAN</t>
+          <t>MANJU CHOUHAN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -812,18 +872,23 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>136.8</v>
+        <v>147.15</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>INV-2026-1015</t>
+          <t>INV-2026-1013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -833,7 +898,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>9413399414</t>
+          <t>9413399464</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -842,18 +907,23 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>307.8</v>
+        <v>317.898</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INV-2026-1016</t>
+          <t>INV-2026-1014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -872,23 +942,28 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>733.5</v>
+        <v>691.6815</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>INV-2026-1017</t>
+          <t>INV-2026-1015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NITESH KUMAR</t>
+          <t>NITISH KUMAR</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -902,9 +977,14 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>19098.2</v>
+        <v>19079.774</v>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -913,7 +993,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>INV-2026-1018</t>
+          <t>INV-2026-1016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -921,20 +1001,21 @@
           <t>ANJANA ASHOK</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>9414064461</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>09-01-2026</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>23778.52</v>
+        <v>24544.47</v>
       </c>
       <c r="F17" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -943,7 +1024,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INV-2026-1019</t>
+          <t>INV-2026-1017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -951,20 +1032,21 @@
           <t>VINOD KUMAR MEENA</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>9772781145</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>09-01-2026</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>12528.75</v>
+        <v>12493.11</v>
       </c>
       <c r="F18" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -973,28 +1055,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>INV-2026-1020</t>
+          <t>INV-2026-1018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PUNIT</t>
+          <t>SAROJ DEVI</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>7564858148</t>
+          <t>8005873419</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3600</v>
+        <v>1119.519</v>
       </c>
       <c r="F19" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -1003,17 +1090,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>INV-2026-1021</t>
+          <t>INV-2026-1019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SAROJ DEVI</t>
+          <t>RAKESH KUMAR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>8005873419</t>
+          <t>620733328</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1022,28 +1109,33 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1164.6</v>
+        <v>317.25</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>INV-2026-1022</t>
+          <t>INV-2026-1020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RAKESH KUMAR</t>
+          <t>MAYA CHOUHAN</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>9620733328</t>
+          <t>9205760608</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1052,28 +1144,33 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>318.6</v>
+        <v>1819.899</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>INV-2026-1023</t>
+          <t>INV-2026-1021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MAYA CHAUHAN</t>
+          <t>SURESH MIROTA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>9205760608</t>
+          <t>9166678263</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1082,28 +1179,33 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1918.8</v>
+        <v>1738.53</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>INV-2026-1024</t>
+          <t>INV-2026-1022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SURESH MIROTA</t>
+          <t>AZIZ MOHAMMAD</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>9166678263</t>
+          <t>9983194736</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1112,28 +1214,33 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1738.8</v>
+        <v>982.8539999999999</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>INV-2026-1025</t>
+          <t>INV-2026-1023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AZIZ MOHAMMAD</t>
+          <t>MOHIT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>9983194736</t>
+          <t>8511919192</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1142,18 +1249,23 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1017</v>
+        <v>295.308</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>INV-2026-1026</t>
+          <t>INV-2026-1024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1172,18 +1284,23 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>974.7</v>
+        <v>955.098</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>INV-2026-1027</t>
+          <t>INV-2026-1025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1193,7 +1310,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>9784305340</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1202,23 +1319,28 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1214.1</v>
+        <v>1181.637</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>INV-2026-1028</t>
+          <t>INV-2026-1026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DIVYA  TAILOR</t>
+          <t>DIVYA TAILOR</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1232,95 +1354,119 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>961.2</v>
+        <v>922.806</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>INV-2026-1029</t>
+          <t>INV-2026-1027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ANSHUL</t>
+          <t>JOGINDER SHARMA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>9928423018</t>
+          <t>9024648186</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>544.5</v>
+        <v>414.495</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>INV-2026-1030</t>
+          <t>INV-2026-1028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JOGINDER SHARMA</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>HUKAM CHAND JAIN</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>9782930312</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>222.2</v>
+        <v>215.0145</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>INV-2026-1032</t>
+          <t>INV-2026-1029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HUKAM CHAND JAIN</t>
+          <t>MOHIT</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>9782930312</t>
+          <t>8511919192</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>214.2</v>
+        <v>259.83</v>
       </c>
       <c r="F30" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -1329,17 +1475,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>INV-2026-1033</t>
+          <t>INV-2026-1030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">MOHIT </t>
+          <t>LAKSH CHOUDHARY</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>8511919192</t>
+          <t>7220030000</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1348,178 +1494,204 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>272.7</v>
+        <v>12493.11</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>INV-2026-1034</t>
+          <t>INV-2026-1031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MAMTA KUMARI</t>
+          <t>ASHA SHARMA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>8218534769</t>
+          <t>9983751185</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>621</v>
+        <v>947.3489999999999</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>INV-2026-1035</t>
+          <t>INV-2026-1032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LAKSH CHOUDHARY</t>
+          <t>NANCHI DEVI</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>7220030000</t>
+          <t>7297987798</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>13400</v>
+        <v>381.9690000000001</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>INV-2026-1037</t>
+          <t>INV-2026-1033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NANCHI DEVI</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>7297987798</t>
-        </is>
-      </c>
+          <t>PUNIT</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>19-01-2026</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>407.7</v>
+        <v>168.75</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>INV-2026-1038</t>
+          <t>INV-2026-1034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">ASHA SHARMA </t>
+          <t>VINOD KUMAR MEENA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>9983751185</t>
+          <t>9772781145</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>950.4</v>
+        <v>16214.1225</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>INV-2026-1039</t>
+          <t>INV-2026-1035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DR.ABHISHEK PRAKASH</t>
+          <t>MANISHA VAISHNAV</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>9024648486</t>
+          <t>9782376560</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>180</v>
+        <v>404.8515</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>INV-2026-1041</t>
+          <t>INV-2026-1036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MANISHA VAISHNAV</t>
+          <t>SANTOSH CHAUHAN</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>9782376560</t>
+          <t>7665939662</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1528,28 +1700,33 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>415.8</v>
+        <v>708.9929999999999</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>INV-2026-1042</t>
+          <t>INV-2026-1037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>VINOD KUMAR MEENA</t>
+          <t>KAMLA DEVI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>9772781145</t>
+          <t>7221043652</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1558,9 +1735,14 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>16250.5</v>
+        <v>1561.275</v>
       </c>
       <c r="F38" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -1569,167 +1751,192 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>INV-2026-1043</t>
+          <t>INV-2026-1038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SANTOSH CHAUHAN</t>
+          <t>RAKESH SHARMA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>7665939662</t>
+          <t>9829691816</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>712.8</v>
+        <v>619.6949999999999</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>INV-2026-1044</t>
+          <t>INV-2026-1039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KAMLA DEVI</t>
+          <t>POONAM JAISWAL</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>7221043652</t>
+          <t>8094496111</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1662.3</v>
+        <v>410.04</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>INV-2026-1045</t>
+          <t>INV-2026-1040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>RAKESH SHARMA</t>
+          <t>ESHA KANWAR</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>9829691816</t>
+          <t>9636390342</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>659.7</v>
+        <v>1336.7565</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>INV-2026-1046</t>
+          <t>INV-2026-1041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>POONAM JAISWAL</t>
+          <t>RAMJI KASHYAP</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>8094496111</t>
+          <t>9660471020</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>437.4</v>
+        <v>1756.701</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>INV-2026-1047</t>
+          <t>INV-2026-1042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESHA KANWAR</t>
+          <t>MAINA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>9636390342</t>
+          <t>8559884415</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1450.8</v>
+        <v>165.573</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>INV-2026-1048</t>
+          <t>INV-2026-1043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RAMJI KASHYAP</t>
+          <t>SAVITRI DEVI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>9660471020</t>
+          <t>9672818823</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1738,88 +1945,103 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1744.2</v>
+        <v>547.992</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>INV-2026-1049</t>
+          <t>INV-2026-1044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MAINA</t>
+          <t>MAYAWATI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>8559884415</t>
+          <t>8502817041</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>165.6</v>
+        <v>151.938</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>INV-2026-1050</t>
+          <t>INV-2026-1045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SAVITRI DEVI</t>
+          <t>M P BHUPATI</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>9672818823</t>
+          <t>9887662251</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>574.2</v>
+        <v>2880.954</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>INV-2026-1051</t>
+          <t>INV-2026-1046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MAYAVATI</t>
+          <t>MINI BHUPATI</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>8502817041</t>
+          <t>8890161369</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1828,28 +2050,33 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>152.1</v>
+        <v>3001.95</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INV-2026-1052</t>
+          <t>INV-2026-1047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>M P BHUPATI</t>
+          <t>VISHNU BHUPATI</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>9887662251</t>
+          <t>8890161369</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1858,28 +2085,33 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2998.8</v>
+        <v>253.116</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INV-2026-1053</t>
+          <t>INV-2026-1048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MINI BHUPATI</t>
+          <t>REKHA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>8890161369</t>
+          <t>7976719725</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1888,28 +2120,33 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>3099.6</v>
+        <v>974.259</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INV-2026-1054</t>
+          <t>INV-2026-1049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VISHNU BHUPATI</t>
+          <t>RAHUL BENIWAL</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>8890161369</t>
+          <t>8302958408</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1918,28 +2155,33 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>270</v>
+        <v>624.996</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>INV-2026-1055</t>
+          <t>INV-2026-1050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>REKHA</t>
+          <t>IRFAN ALI</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>7976719725</t>
+          <t>9057549996</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1948,71 +2190,2492 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>976.5</v>
+        <v>1071.495</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>INV-2026-1056</t>
+          <t>INV-2026-1051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RAHUL BENIWAL</t>
+          <t>J B NAG</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>8302958408</t>
+          <t>9007053421</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>623.7</v>
+        <v>621.477</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>ranjeet</t>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>INV-2026-1052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>GAURAV KUMAR</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7014894823</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>27-01-2026</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>512.7624999999999</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>INV-2026-1053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>GAURAV KUMAR</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7014894823</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>27-01-2026</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>576.7199999999999</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>INV-2026-1054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AJAY MADHIWAL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>7976401116</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>27-01-2026</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1599.966</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>INV-2026-1055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>MRS SONALI GUPTA</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>9309400500</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>27-01-2026</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>402.228</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>INV-2026-1056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>MR ASHU MATHUR</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>9423637256</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>28-01-2026</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>913.7070000000001</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>INV-2026-1057</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>IRFAN ALI</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>9057549996</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>26-01-2026</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>1113.3</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>ranjeet</t>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>JAWAHAR LAL KAUL</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>9357405038</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>28-01-2026</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>197.613</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>INV-2026-1058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>NIDHI JAIN</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>8638654822</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>29-01-2026</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>190.143</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>INV-2026-1059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>STUTI JAIN</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>8851479583</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>29-01-2026</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1002.231</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>INV-2026-1060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SOMAL SHRUTI</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>9611586003</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>29-01-2026</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>126.126</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>INV-2026-1061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>RAJESH SONAWANE</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>996041460</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>30-01-2026</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>310.419</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>INV-2026-1062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>MISS TRISHA</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>9982169332</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>30-01-2026</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>728.973</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>INV-2026-1063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>MRS SUMITRA</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>7820999955</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>31-01-2026</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1515.915</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>INV-2026-1064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>INDRA JOSHI</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>7073453834</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>31-01-2026</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>344.628</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>INV-2026-1065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>MRS SURAJ BAI</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>8657663957</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>31-01-2026</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>126.558</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>INV-2026-1066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>MR NARENDRA KUMAR</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>9986049566</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>865.9440000000001</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>INV-2026-1067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>MRS UMA DEVI</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>7850081952</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>350.676</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>INV-2026-1068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>MR HUKAM CHAND JAIN</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>9782930312</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>133.389</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>INV-2026-1069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>MRS RASHMI KHATRI</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>998333996</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>677.277</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>INV-2026-1070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>JAWAHAR LAL KAUL</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>9357405038</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1140.66</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>INV-2026-1071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SURGYAN RAYKA</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>6378299639</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>326.25</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>INV-2026-1072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>RACHNA SAINI</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>9799887771</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1490.325</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>INV-2026-1073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ANKIT KAKKAR</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>9171951444</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>672.732</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>INV-2026-1074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SURBHI KAKKAD</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>8171951444</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>637.335</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>INV-2026-1075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SUBASH CHAND</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>405.684</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>INV-2026-1076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>SUMITRA SAINI</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>6204987554</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>362.799</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>INV-2026-1077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SHILPI</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>7023939797</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1401.228</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>INV-2026-1078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>JASMIT KAUR</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>9784596838</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>02-02-2026</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>430.029</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>INV-2026-1079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SURBHI KAKKAD</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>8171951444</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>168.912</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>INV-2026-1080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>LEELA FULWANI</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>9167706038</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1114.56</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>INV-2026-1081</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>RAKESH SHARMA</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>9829691816</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1592.649</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>INV-2026-1082</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MR HUKAM CHAND JAIN</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>9782930312</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>627.0435</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>INV-2026-1083</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MR GNAPAT RAJVASNSHI</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>8955520922</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1676.484</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>INV-2026-1084</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SURBHI KAKKAD</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>8171951444</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>337.662</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>INV-2026-1085</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MR MAHENDRA SINGH</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>8769980558</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1156.383</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>INV-2026-1086</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MISS SURBHI MEENA</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>9680926505</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>12725.628</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>INV-2026-1087</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SUSHMITA KUDU</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>9057823252</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2798.946</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>INV-2026-1088</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MR RAJENDRA KUMAR</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>7014852038</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>06-02-2026</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1050.32</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>INV-2026-1089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MRS BHARTI SHARMA</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>8233094519</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>870.408</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>INV-2026-1090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MRS MAMTA JAIN</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>9829147353</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>07-02-2026</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>143.1</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>INV-2026-1091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>MRS MOHINI</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>7823808585</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>07-02-2026</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>597.744</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>INV-2026-1092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>MR GAURAV SHARMA</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>7014894823</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>07-02-2026</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1544.028</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>INV-2026-1093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>MRS RUCHI JAIN</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>9694547045</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>07-02-2026</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>512.073</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>INV-2026-1094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>MRS NISHA KUMARI</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>8094014597</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>10-02-2026</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>1291.356</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>INV-2026-1095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MRS SANGEETA SHARMA</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>8708285527</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>191.52</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>INV-2026-1096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>SEEMA SANTORIA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>9474538263</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>11-02-2026</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>570.087</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>INV-2026-1097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>NISHA TULSIAN</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>9351547222</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>11-02-2026</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>39.86199999999999</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>INV-2026-1098</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>VIKASH</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1063.692</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>INV-2026-1099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>LAJWANTI KHATRI</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>583.875</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>INV-2026-1100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>VINOD KUMAR MEENA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>9772781145</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>15638.4575</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>INV-2026-1101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MRS PRIYANKA JOSHI</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>8118876991</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>8849.32</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>INV-2026-1102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SAROJ DEVI</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>281.808</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>INV-2026-1103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>ANURAG CHOUDHARY</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>79.72399999999999</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>INV-2026-1104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SUSHMITA SAINI</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>8078671687</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>1325.997</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>INV-2026-1105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>RAJENDRA</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>8875678277</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>871.173</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>INV-2026-1106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MADHU KUMAWAT</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>9079366613</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1515.474</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>INV-2026-1107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SURBHI SHARMA</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>9819308057</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>13-02-2026</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>340.6545</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>INV-2026-1108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>MADHURI</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>8003010101</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>14-02-2026</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>194.967</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>INV-2026-1109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>AKSHAT GOYAL</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>7357503800</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>14-02-2026</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>574.605</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>INV-2026-1110</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>RASHMI</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>16-02-2026</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1911.555</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>INV-2026-1111</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>JAY SONI</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>6204987554</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>18-02-2026</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>382.86</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>INV-2026-1112</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SUMAN SHRIVASTAV</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>16-02-2026</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>1156.851</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>INV-2026-1113</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>RIYA SHARMA</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>16-02-2026</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1357.119</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>INV-2026-1114</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>RADHA KANVAR</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>16-02-2026</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>444.2130000000001</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>INV-2026-1115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>YASH CHOUDHARY</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>16-02-2026</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>797.499</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>INV-2026-1116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>PUNIT</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>16-02-2026</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>621.5309999999999</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>INV-2026-1117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>MAMTA KUMARI</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>8218534769</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>16-01-2026</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>620.64</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>INV-2026-1118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>LAJWANTI KHATRI</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>8058614558</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>30-01-2026</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>529.779</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>INV-2026-1119</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>VIRENDRA KUMAR ARYA</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>9314685876</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>30-01-2026</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>413.76</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>INV-2026-1120</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>MR MAHESH MULEY</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>9922273906</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>30-01-2026</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>1103.934</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>INV-2026-1121</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>MR ARCHNA GOYAL</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>9664047073</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>19-02-2026</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1082.544</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>INV-2026-1122</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>MRS RASHMI KHATRI</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>9983333996</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>19-02-2026</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>140.904</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>admin</t>
         </is>
       </c>
     </row>

</xml_diff>